<commit_message>
Add S6M marketing campaign wizard (slices 6M-0 through 6M-4).
Introduces campaign-centric marketing with draft wizard, recipients, template library/composer, and multi-step email sequences so the redesign can be validated on preview before production launch.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/FlowChat_User_Stories_S1_S6.xlsx
+++ b/FlowChat_User_Stories_S1_S6.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K149"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3566,15 +3566,12 @@
         <v>Must</v>
       </c>
       <c r="J82" t="str">
-        <v>Completed</v>
+        <v>Superseded</v>
       </c>
       <c r="K82" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Workflow builder shows a visual step canvas with drag-to-add nodes
-• Triggers available: contact created, label added, conversation resolved, manual enroll
-• Actions available: send email (pick template), wait (hours/days), branch (if opened / if clicked / else), add label, exit workflow
-• Published workflow enrolls matching contacts automatically
-• Workflow can be paused and resumed; enrolled contacts retain their position
-• Workflow dashboard shows enrolled count, completed count, and step-level stats</v>
+        <v xml:space="preserve">• [Superseded by S6M — see marketing-module-screens.md] Was: visual workflow builder with CRM triggers (contact created, label added, conversation resolved)
+• Replacement: campaign-only wizard with explicit recipients (S6M-6, S6M-9)
+• Remove triggerMarketingWorkflows at S6M-9 implementation</v>
       </c>
     </row>
     <row r="83" xml:space="preserve">
@@ -3606,14 +3603,11 @@
         <v>Must</v>
       </c>
       <c r="J83" t="str">
-        <v>Completed</v>
+        <v>Superseded</v>
       </c>
       <c r="K83" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Drip sequence is a series of wait + send email steps within a workflow
-• Each wait step supports delay in hours or days
-• Enrollment cap limits the total number of contacts in the workflow at once
-• Re-entry rules: once only, or allow re-enroll after N days
-• Contact's current step is visible on the workflow enrollment list</v>
+        <v xml:space="preserve">• [Superseded by S6M] Was: multi-step drip inside CRM-triggered workflows
+• Replacement: multi-step dated campaign sequence in wizard (S6M-16–S6M-18)</v>
       </c>
     </row>
     <row r="84" xml:space="preserve">
@@ -4076,360 +4070,2009 @@
     </row>
     <row r="96" xml:space="preserve">
       <c r="A96" t="str">
+        <v>S6M-1</v>
+      </c>
+      <c r="B96" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Campaign lifecycle</v>
+      </c>
+      <c r="F96" t="str">
+        <v>As a Sales agent, I want to create a marketing campaign draft that receives a campaign ID immediately, so that I can save progress and return later.</v>
+      </c>
+      <c r="G96" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H96">
+        <v>5</v>
+      </c>
+      <c r="I96" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J96" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K96" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Wizard step 0 saves draft via POST /marketing/campaigns
+• Response includes campaign id displayed in UI
+• Draft persists name, owner, created_at
+• Deep link /marketing/campaigns/:id/edit?step=N resumes wizard</v>
+      </c>
+    </row>
+    <row r="97" xml:space="preserve">
+      <c r="A97" t="str">
+        <v>S6M-2</v>
+      </c>
+      <c r="B97" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Campaign lifecycle</v>
+      </c>
+      <c r="F97" t="str">
+        <v>As a Sales agent, I want a campaigns list with status filters, so that I can find drafts, running, and completed outreach.</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H97">
+        <v>3</v>
+      </c>
+      <c r="I97" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J97" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K97" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Marketing home lists campaigns with status badges: draft, scheduled, running, paused, completed, cancelled
+• Filter by status and search by name
+• Shows recipient count and next scheduled send</v>
+      </c>
+    </row>
+    <row r="98" xml:space="preserve">
+      <c r="A98" t="str">
+        <v>S6M-3</v>
+      </c>
+      <c r="B98" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Campaign lifecycle</v>
+      </c>
+      <c r="F98" t="str">
+        <v>As an Admin, I want to launch a campaign after review, so that scheduled emails begin processing in the background.</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="H98">
+        <v>5</v>
+      </c>
+      <c r="I98" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J98" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K98" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Only administrator role can launch
+• Launch validates pre-flight checks (provider, test send, recipients)
+• Status moves draft → scheduled/running
+• Background job enqueues step 1 per recipient
+• Audit: launched_by user id + launched_at timestamp stored on campaign; shown on stats header</v>
+      </c>
+    </row>
+    <row r="99" xml:space="preserve">
+      <c r="A99" t="str">
+        <v>S6M-4</v>
+      </c>
+      <c r="B99" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Campaign lifecycle</v>
+      </c>
+      <c r="F99" t="str">
+        <v>As an Admin, I want to pause or cancel a running campaign, so that no further steps send until I decide.</v>
+      </c>
+      <c r="G99" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="H99">
+        <v>3</v>
+      </c>
+      <c r="I99" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J99" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K99" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Pause stops new sends; in-flight batch completes
+• Cancel marks campaign cancelled; pending recipient steps skipped
+• Confirmation modals show recipient impact summary (§4.10 marketing-module-screens.md)
+• Activity log records pause/cancel events</v>
+      </c>
+    </row>
+    <row r="100" xml:space="preserve">
+      <c r="A100" t="str">
+        <v>S6M-5</v>
+      </c>
+      <c r="B100" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Campaign lifecycle</v>
+      </c>
+      <c r="F100" t="str">
+        <v>As a Sales agent, I want to duplicate a completed campaign as a new draft, so that I can repeat outreach with a new schedule.</v>
+      </c>
+      <c r="G100" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H100">
+        <v>3</v>
+      </c>
+      <c r="I100" t="str">
+        <v>Should</v>
+      </c>
+      <c r="J100" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K100" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Duplicate copies steps and templates (snapshot) not live template links
+• Recipients not copied; test-send and launch audit reset
+• New campaign id assigned; redirect to edit step 2 to reschedule (§4.11 marketing-module-screens.md)</v>
+      </c>
+    </row>
+    <row r="101" xml:space="preserve">
+      <c r="A101" t="str">
+        <v>S6M-6</v>
+      </c>
+      <c r="B101" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Recipients</v>
+      </c>
+      <c r="F101" t="str">
+        <v>As a Sales agent, I want to select multiple email recipients in the campaign wizard, so that only chosen contacts receive the sequence.</v>
+      </c>
+      <c r="G101" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H101">
+        <v>5</v>
+      </c>
+      <c r="I101" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J101" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K101" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Step 1: search CRM contacts with email
+• Multi-select with select-all on page
+• At least one recipient required to proceed
+• Selected count shown on review step</v>
+      </c>
+    </row>
+    <row r="102" xml:space="preserve">
+      <c r="A102" t="str">
+        <v>S6M-7</v>
+      </c>
+      <c r="B102" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Recipients</v>
+      </c>
+      <c r="F102" t="str">
+        <v>As a Sales agent, I want to load recipients from a static segment, so that I can reuse a campaign list without auto-emailing new CRM contacts.</v>
+      </c>
+      <c r="G102" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H102">
+        <v>3</v>
+      </c>
+      <c r="I102" t="str">
+        <v>Should</v>
+      </c>
+      <c r="J102" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K102" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Optional “Import from segment” on step 1
+• Merges segment members into selection; user can deselect individuals
+• Dynamic segments show preview count before import</v>
+      </c>
+    </row>
+    <row r="103" xml:space="preserve">
+      <c r="A103" t="str">
+        <v>S6M-8</v>
+      </c>
+      <c r="B103" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Recipients</v>
+      </c>
+      <c r="F103" t="str">
+        <v>As a Sales agent, I want warnings for suppressed or invalid recipients, so that I do not accidentally include bounced or unsubscribed contacts.</v>
+      </c>
+      <c r="G103" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H103">
+        <v>3</v>
+      </c>
+      <c r="I103" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J103" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K103" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Suppressed/unsubscribed/bounced contacts flagged in picker
+• Launch blocks sends to suppressed addresses
+• Summary shows excluded count with reasons</v>
+      </c>
+    </row>
+    <row r="104" xml:space="preserve">
+      <c r="A104" t="str">
+        <v>S6M-9</v>
+      </c>
+      <c r="B104" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E104" t="str">
+        <v>CRM isolation</v>
+      </c>
+      <c r="F104" t="str">
+        <v>As a Platform, I want no marketing email triggered on contact create/import/chat, so that outreach only starts from the Marketing module.</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H104">
+        <v>5</v>
+      </c>
+      <c r="I104" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J104" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K104" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Remove triggerMarketingWorkflows on contact_created from: manual CRUD, CSV import, LeadSnapper/integration upsert, widget session create
+• Remove conversation_resolved and label_added auto-enroll from marketing
+• Legacy workflow UI hidden or admin-only deprecated
+• CRM contacts unaffected when added via any medium; double opt-in transactional mail is not a marketing campaign</v>
+      </c>
+    </row>
+    <row r="105" xml:space="preserve">
+      <c r="A105" t="str">
+        <v>S6M-10</v>
+      </c>
+      <c r="B105" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Recipients</v>
+      </c>
+      <c r="F105" t="str">
+        <v>As a Sales agent, I want a review step showing all recipients before launch, so that I can confirm the audience.</v>
+      </c>
+      <c r="G105" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H105">
+        <v>2</v>
+      </c>
+      <c r="I105" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J105" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K105" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Step 4 lists recipient names and emails (paginated)
+• Shows subscribed-only confirmation
+• Edit recipients link returns to step 1</v>
+      </c>
+    </row>
+    <row r="106" xml:space="preserve">
+      <c r="A106" t="str">
+        <v>S6M-11</v>
+      </c>
+      <c r="B106" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Templates</v>
+      </c>
+      <c r="F106" t="str">
+        <v>As a Sales agent, I want a template library independent of campaigns, so that I can build reusable email content ahead of time.</v>
+      </c>
+      <c r="G106" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H106">
+        <v>5</v>
+      </c>
+      <c r="I106" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J106" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K106" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Marketing → Templates: list, create, edit, archive, duplicate
+• Templates have name, subject, html_body, plain text fallback auto-generated from HTML on save (editable)
+• No campaign required to save a template</v>
+      </c>
+    </row>
+    <row r="107" xml:space="preserve">
+      <c r="A107" t="str">
+        <v>S6M-12</v>
+      </c>
+      <c r="B107" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Templates</v>
+      </c>
+      <c r="F107" t="str">
+        <v>As a Sales agent, I want a full-screen enterprise email composer, so that I can write professional HTML emails with focus.</v>
+      </c>
+      <c r="G107" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H107">
+        <v>8</v>
+      </c>
+      <c r="I107" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J107" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K107" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Composer opens full viewport overlay from wizard or template library
+• Rich text: headings, bold, links, lists, undo
+• Subject line field above body
+• Mobile-safe preview toggle
+• Escape/minimize returns to wizard without losing draft</v>
+      </c>
+    </row>
+    <row r="108" xml:space="preserve">
+      <c r="A108" t="str">
+        <v>S6M-13</v>
+      </c>
+      <c r="B108" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Templates</v>
+      </c>
+      <c r="F108" t="str">
+        <v>As a Sales agent, I want a checkbox to save an email as a template during the campaign wizard, so that I can reuse content on future campaigns.</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H108">
+        <v>3</v>
+      </c>
+      <c r="I108" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J108" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K108" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Per sequence step: “Save as template” with name field
+• On launch, creates template if checked
+• Template library shows source campaign metadata optional</v>
+      </c>
+    </row>
+    <row r="109" xml:space="preserve">
+      <c r="A109" t="str">
+        <v>S6M-14</v>
+      </c>
+      <c r="B109" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Templates</v>
+      </c>
+      <c r="F109" t="str">
+        <v>As a Platform, I want campaign email content snapshotted at launch, so that later template edits do not change in-flight campaigns.</v>
+      </c>
+      <c r="G109" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H109">
+        <v>3</v>
+      </c>
+      <c r="I109" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J109" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K109" t="str" xml:space="preserve">
+        <v xml:space="preserve">• campaign_steps store subject/html snapshot per step
+• Editing library template does not alter running campaign
+• Duplicate campaign copies snapshots</v>
+      </c>
+    </row>
+    <row r="110" xml:space="preserve">
+      <c r="A110" t="str">
+        <v>S6M-15</v>
+      </c>
+      <c r="B110" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Templates</v>
+      </c>
+      <c r="F110" t="str">
+        <v>As a Sales agent, I want merge tag chips in the composer, so that I can insert personalization tokens without typing syntax.</v>
+      </c>
+      <c r="G110" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H110">
+        <v>5</v>
+      </c>
+      <c r="I110" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J110" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K110" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Chips: first_name, last_name, email, phone, contact_message, meeting_link, portfolio_link, agent_name, agent_email
+• Insert at cursor in subject or body
+• Preview mode renders sample contact</v>
+      </c>
+    </row>
+    <row r="111" xml:space="preserve">
+      <c r="A111" t="str">
+        <v>S6M-16</v>
+      </c>
+      <c r="B111" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Email sequence</v>
+      </c>
+      <c r="F111" t="str">
+        <v>As a Sales agent, I want to add multiple follow-up emails in one campaign, so that I can run dated sequences.</v>
+      </c>
+      <c r="G111" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H111">
+        <v>5</v>
+      </c>
+      <c r="I111" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J111" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K111" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Step 2: add/remove email rows (min 1)
+• Each row: pick one template or write from scratch
+• Optional bulk apply: select multiple templates at once → creates one step per template with default schedule spacing
+• Sequence order preserved as step_order</v>
+      </c>
+    </row>
+    <row r="112" xml:space="preserve">
+      <c r="A112" t="str">
+        <v>S6M-17</v>
+      </c>
+      <c r="B112" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Email sequence</v>
+      </c>
+      <c r="F112" t="str">
+        <v>As a Sales agent, I want to set an explicit date and time for each email, so that scheduling is fully under my control.</v>
+      </c>
+      <c r="G112" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H112">
+        <v>5</v>
+      </c>
+      <c r="I112" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J112" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K112" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Date+time picker per step; no system timezone preference for scheduling UI
+• Display shows agent-selected datetime as stored (UTC backend)
+• Timeline preview visualizes all steps</v>
+      </c>
+    </row>
+    <row r="113" xml:space="preserve">
+      <c r="A113" t="str">
+        <v>S6M-18</v>
+      </c>
+      <c r="B113" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Email sequence</v>
+      </c>
+      <c r="F113" t="str">
+        <v>As a Sales agent, I want validation that each follow-up is scheduled after the previous email, so that the sequence order is logical.</v>
+      </c>
+      <c r="G113" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H113">
+        <v>3</v>
+      </c>
+      <c r="I113" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J113" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K113" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Step N send_at &gt; step N-1 send_at
+• All send_at must be in the future at launch
+• Clear inline error on violation</v>
+      </c>
+    </row>
+    <row r="114" xml:space="preserve">
+      <c r="A114" t="str">
+        <v>S6M-19</v>
+      </c>
+      <c r="B114" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Email sequence</v>
+      </c>
+      <c r="F114" t="str">
+        <v>As a Sales agent, I want to pick a contact message for the contact_message merge field, so that emails reference a specific note or chat message.</v>
+      </c>
+      <c r="G114" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H114">
+        <v>5</v>
+      </c>
+      <c r="I114" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J114" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K114" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Per step with {{contact_message}}: agent selects source mode (industry-standard per-recipient resolution):
+  – latest_note: most recent CRM note for each recipient
+  – latest_inbound_chat: most recent visitor message in any linked conversation
+  – latest_note_or_chat: inbound chat if any, else latest note, else omit token
+• Wizard preview uses sample contact (first selected recipient or explicit sample picker); send-time resolution is per recipient
+• merge_config stored on campaign_step; empty resolution omits token (no literal placeholder)
+• Source mode required before launch when token present</v>
+      </c>
+    </row>
+    <row r="115" xml:space="preserve">
+      <c r="A115" t="str">
+        <v>S6M-20</v>
+      </c>
+      <c r="B115" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Email sequence</v>
+      </c>
+      <c r="F115" t="str">
+        <v>As a Platform, I want file attachments disabled in marketing emails, so that campaigns stay lightweight and compliant.</v>
+      </c>
+      <c r="G115" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H115">
+        <v>2</v>
+      </c>
+      <c r="I115" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J115" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K115" t="str" xml:space="preserve">
+        <v xml:space="preserve">• No attachment UI in composer
+• API rejects attachment payloads on campaign send
+• QA checklist includes negative test</v>
+      </c>
+    </row>
+    <row r="116" xml:space="preserve">
+      <c r="A116" t="str">
+        <v>S6M-21</v>
+      </c>
+      <c r="B116" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Signature &amp; compliance</v>
+      </c>
+      <c r="F116" t="str">
+        <v>As a Sales agent, I want a proper signature block after my name in the footer, so that emails look professional.</v>
+      </c>
+      <c r="G116" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H116">
+        <v>5</v>
+      </c>
+      <c r="I116" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J116" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K116" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Step 3: signature rich editor or workspace default
+• Rendered after body: agent name → signature HTML
+• Validation: signature or workspace default required</v>
+      </c>
+    </row>
+    <row r="117" xml:space="preserve">
+      <c r="A117" t="str">
+        <v>S6M-22</v>
+      </c>
+      <c r="B117" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Signature &amp; compliance</v>
+      </c>
+      <c r="F117" t="str">
+        <v>As a Sales agent, I want meeting and portfolio links in the footer, so that recipients can book or view our work.</v>
+      </c>
+      <c r="G117" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H117">
+        <v>3</v>
+      </c>
+      <c r="I117" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J117" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K117" t="str" xml:space="preserve">
+        <v xml:space="preserve">• meeting_link and portfolio_link merge tags from workspace settings; overridable per campaign
+• Appended in footer block after signature
+• Preview shows resolved URLs</v>
+      </c>
+    </row>
+    <row r="118" xml:space="preserve">
+      <c r="A118" t="str">
+        <v>S6M-23</v>
+      </c>
+      <c r="B118" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Signature &amp; compliance</v>
+      </c>
+      <c r="F118" t="str">
+        <v>As a Sales agent, I must send a test email before an admin launches the campaign, so that content and deliverability are verified.</v>
+      </c>
+      <c r="G118" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H118">
+        <v>5</v>
+      </c>
+      <c r="I118" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J118" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K118" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Launch button disabled until a test send succeeded for this campaign draft (persists across sessions until content/sender changes invalidate)
+• Agent or admin can trigger test; uses step 1 content with logged-in user as merge sample
+• Test send logged on campaign: test_sent_at, test_sent_by, test_sent_to; invalidates if step 1 subject/body or sender changes</v>
+      </c>
+    </row>
+    <row r="119" xml:space="preserve">
+      <c r="A119" t="str">
+        <v>S6M-24</v>
+      </c>
+      <c r="B119" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Infrastructure</v>
+      </c>
+      <c r="F119" t="str">
+        <v>As an Admin, I want a pre-flight panel showing email provider and cron health, so that I know the system can send before launch.</v>
+      </c>
+      <c r="G119" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="H119">
+        <v>5</v>
+      </c>
+      <c r="I119" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J119" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K119" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Checks: connected Resend/SendGrid/Mailgun or platform key; domain verified; last cron success &lt; 2 min
+• Failures show actionable messages
+• Shown on review step and Settings → Email marketing</v>
+      </c>
+    </row>
+    <row r="120" xml:space="preserve">
+      <c r="A120" t="str">
+        <v>S6M-25</v>
+      </c>
+      <c r="B120" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Signature &amp; compliance</v>
+      </c>
+      <c r="F120" t="str">
+        <v>As a Platform, I want unsubscribe and physical address footer on every marketing email, so that we stay compliant.</v>
+      </c>
+      <c r="G120" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H120">
+        <v>3</v>
+      </c>
+      <c r="I120" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J120" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K120" t="str" xml:space="preserve">
+        <v xml:space="preserve">• System appends List-Unsubscribe header and footer link
+• Physical address from workspace settings
+• Cannot be removed by agent; preview shows footer</v>
+      </c>
+    </row>
+    <row r="121" xml:space="preserve">
+      <c r="A121" t="str">
+        <v>S6M-26</v>
+      </c>
+      <c r="B121" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Analytics</v>
+      </c>
+      <c r="F121" t="str">
+        <v>As a Sales agent, I want a campaign overview with funnel metrics, so that I see performance at a glance.</v>
+      </c>
+      <c r="G121" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H121">
+        <v>5</v>
+      </c>
+      <c r="I121" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J121" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K121" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Detail page: sent, delivered, opened, clicked, bounced, unsubscribed, complained, stopped counts
+• Aggregate open/click rates
+• Live progress during running state
+• Activity log tab: chronological send attempts, webhook events, skips, sanitized errors (admin-readable)</v>
+      </c>
+    </row>
+    <row r="122" xml:space="preserve">
+      <c r="A122" t="str">
+        <v>S6M-27</v>
+      </c>
+      <c r="B122" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E122" t="str">
+        <v>Analytics</v>
+      </c>
+      <c r="F122" t="str">
+        <v>As a Sales agent, I want per-email-step statistics, so that I know which follow-up performs best.</v>
+      </c>
+      <c r="G122" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H122">
+        <v>5</v>
+      </c>
+      <c r="I122" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J122" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K122" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Tab or section per step: subject, scheduled time, sent count, open %, click %
+• Stopped-by-bounce/reply/unsub/complaint counts per step</v>
+      </c>
+    </row>
+    <row r="123" xml:space="preserve">
+      <c r="A123" t="str">
+        <v>S6M-28</v>
+      </c>
+      <c r="B123" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E123" t="str">
+        <v>Analytics</v>
+      </c>
+      <c r="F123" t="str">
+        <v>As a Sales agent, I want a recipient table with filters, so that I can see who opened, clicked, or stopped.</v>
+      </c>
+      <c r="G123" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H123">
+        <v>5</v>
+      </c>
+      <c r="I123" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J123" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K123" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Columns: contact, email, per-step status, stopped_reason, last event time
+• Filters: opened, not_opened, clicked, bounced, stopped_bounce, stopped_unsubscribe, stopped_reply, stopped_complaint (map from campaign_recipient.stopped_reason per §1.2 in marketing-module-screens.md)
+• Link to contact profile</v>
+      </c>
+    </row>
+    <row r="124" xml:space="preserve">
+      <c r="A124" t="str">
+        <v>S6M-29</v>
+      </c>
+      <c r="B124" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E124" t="str">
+        <v>Analytics</v>
+      </c>
+      <c r="F124" t="str">
+        <v>As an Admin, I want to export campaign results as CSV, so that I can report offline.</v>
+      </c>
+      <c r="G124" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="H124">
+        <v>3</v>
+      </c>
+      <c r="I124" t="str">
+        <v>Should</v>
+      </c>
+      <c r="J124" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K124" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Export recipient × step × status × timestamps
+• Includes stopped_reason column
+• Download from campaign detail</v>
+      </c>
+    </row>
+    <row r="125" xml:space="preserve">
+      <c r="A125" t="str">
+        <v>S6M-30</v>
+      </c>
+      <c r="B125" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E125" t="str">
+        <v>Analytics</v>
+      </c>
+      <c r="F125" t="str">
+        <v>As a Sales agent, I want campaign emails on the contact profile timeline, so that CRM and marketing stay connected.</v>
+      </c>
+      <c r="G125" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H125">
+        <v>3</v>
+      </c>
+      <c r="I125" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J125" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K125" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Contact profile shows campaign name, step, sent/opened/clicked/stopped events
+• Consistent with campaign detail recipient row</v>
+      </c>
+    </row>
+    <row r="126" xml:space="preserve">
+      <c r="A126" t="str">
+        <v>S6M-31</v>
+      </c>
+      <c r="B126" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E126" t="str">
+        <v>Infrastructure</v>
+      </c>
+      <c r="F126" t="str">
+        <v>As a Platform, I want try/catch and safe error messages across the marketing module, so that failures never expose raw provider responses.</v>
+      </c>
+      <c r="G126" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H126">
+        <v>5</v>
+      </c>
+      <c r="I126" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J126" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K126" t="str" xml:space="preserve">
+        <v xml:space="preserve">• MarketingError codes mapped to UI strings per §3.1 marketing-module-screens.md
+• API returns { error, code }; no stack traces to client
+• Failed sends retried with cap; logged server-side</v>
+      </c>
+    </row>
+    <row r="127" xml:space="preserve">
+      <c r="A127" t="str">
+        <v>S6M-32</v>
+      </c>
+      <c r="B127" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E127" t="str">
+        <v>Infrastructure</v>
+      </c>
+      <c r="F127" t="str">
+        <v>As an Admin, I want only administrators to launch campaigns, so that outbound email is controlled.</v>
+      </c>
+      <c r="G127" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="H127">
+        <v>3</v>
+      </c>
+      <c r="I127" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J127" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K127" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Agents can build drafts; launch requires administrator role
+• API enforces RBAC on launch/pause/cancel
+• Agents on step 4 see info banner: “An administrator must launch this campaign” + Launch button hidden; test send and Save draft remain available</v>
+      </c>
+    </row>
+    <row r="128" xml:space="preserve">
+      <c r="A128" t="str">
+        <v>S6M-33</v>
+      </c>
+      <c r="B128" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E128" t="str">
+        <v>Infrastructure</v>
+      </c>
+      <c r="F128" t="str">
+        <v>As a Platform, I want the cron/worker to process campaign steps by scheduled time, so that follow-ups send reliably in the background.</v>
+      </c>
+      <c r="G128" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H128">
+        <v>8</v>
+      </c>
+      <c r="I128" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J128" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K128" t="str" xml:space="preserve">
+        <v xml:space="preserve">• job-runner processes campaign_recipient_steps where send_at &lt;= now
+• Idempotent: same step+recipient never double-sent
+• Primary: Railway worker polls GET /api/cron/marketing every ~60s
+• Backup: Vercel Cron hits same endpoint every 5 min when WORKER unavailable (env + runbook documented)
+• Health panel shows last successful cron timestamp</v>
+      </c>
+    </row>
+    <row r="129" xml:space="preserve">
+      <c r="A129" t="str">
+        <v>S6M-34</v>
+      </c>
+      <c r="B129" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E129" t="str">
+        <v>Infrastructure</v>
+      </c>
+      <c r="F129" t="str">
+        <v>As a Platform, I want delivery webhooks from Resend/SendGrid/Mailgun to update stats, so that opens and bounces reflect within minutes.</v>
+      </c>
+      <c r="G129" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H129">
+        <v>5</v>
+      </c>
+      <c r="I129" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J129" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K129" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Per-credential webhook URLs ingest delivered, opened, clicked, bounced, complained
+• Updates campaign_recipient_step status and contact_email_events
+• Webhook signature verified</v>
+      </c>
+    </row>
+    <row r="130" xml:space="preserve">
+      <c r="A130" t="str">
+        <v>S6M-35</v>
+      </c>
+      <c r="B130" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C130" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E130" t="str">
+        <v>CRM isolation</v>
+      </c>
+      <c r="F130" t="str">
+        <v>As an Admin, I want legacy CRM-triggered workflows removed from Marketing navigation, so that agents only use the campaign wizard.</v>
+      </c>
+      <c r="G130" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="H130">
+        <v>3</v>
+      </c>
+      <c r="I130" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J130" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K130" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Nav: Campaigns, Templates only (segments optional sub-link)
+• /marketing/workflows and old automations redirect or 410
+• Docs updated</v>
+      </c>
+    </row>
+    <row r="131" xml:space="preserve">
+      <c r="A131" t="str">
+        <v>S6M-36</v>
+      </c>
+      <c r="B131" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C131" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E131" t="str">
+        <v>Stop rules</v>
+      </c>
+      <c r="F131" t="str">
+        <v>As a Platform, I want hard bounces to stop all remaining follow-ups for that recipient in the campaign, so that we do not mail invalid addresses.</v>
+      </c>
+      <c r="G131" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H131">
+        <v>5</v>
+      </c>
+      <c r="I131" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J131" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K131" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Hard/permanent bounce (provider permanent flag or second soft within 72h): campaign_recipient.stopped_reason=bounce; pending steps set status=stopped_bounce
+• Soft bounce: retry once after 4h; second failure treated as hard bounce
+• Global suppress on hard bounce (contact email status)
+• Other recipients continue
+• Stats aggregate stopped_bounce count</v>
+      </c>
+    </row>
+    <row r="132" xml:space="preserve">
+      <c r="A132" t="str">
+        <v>S6M-37</v>
+      </c>
+      <c r="B132" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C132" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E132" t="str">
+        <v>Stop rules</v>
+      </c>
+      <c r="F132" t="str">
+        <v>As a Platform, I want unsubscribes to stop all remaining follow-ups for that email address in the campaign, so that opt-out is honoured immediately.</v>
+      </c>
+      <c r="G132" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H132">
+        <v>3</v>
+      </c>
+      <c r="I132" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J132" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K132" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Unsubscribe link suppresses globally and stops pending campaign steps for that address
+• campaign_recipient.stopped_reason=unsubscribe; pending steps status=stopped_unsubscribe
+• Launch already blocks suppressed addresses</v>
+      </c>
+    </row>
+    <row r="133" xml:space="preserve">
+      <c r="A133" t="str">
+        <v>S6M-38</v>
+      </c>
+      <c r="B133" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E133" t="str">
+        <v>Stop rules</v>
+      </c>
+      <c r="F133" t="str">
+        <v>As a Platform, I want replies from the recipient email address to stop remaining follow-ups in that campaign, so that engaged contacts are not over-mailed.</v>
+      </c>
+      <c r="G133" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H133">
+        <v>8</v>
+      </c>
+      <c r="I133" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J133" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K133" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Primary: inbound reply matched via In-Reply-To/References to outbound Message-ID (Sprint 7 email inbox)
+• Fallback until inbox live: provider reply/engagement webhook if supported by connected ESP
+• campaign_recipient.stopped_reason=reply; pending steps status=stopped_reply
+• Reply does not stop other campaigns or other recipients
+• Documented dependency: full reply-stop requires Sprint 7 inbound routing</v>
+      </c>
+    </row>
+    <row r="134" xml:space="preserve">
+      <c r="A134" t="str">
+        <v>S6M-39</v>
+      </c>
+      <c r="B134" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E134" t="str">
+        <v>Campaign lifecycle</v>
+      </c>
+      <c r="F134" t="str">
+        <v>As a Sales agent, I want wizard step navigation with saved progress, so that I can complete a campaign across sessions.</v>
+      </c>
+      <c r="G134" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H134">
+        <v>5</v>
+      </c>
+      <c r="I134" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J134" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K134" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Steps: Recipients → Sequence → Sender → Review
+• Back/next preserves data; autosave on step change
+• Invalid step cannot proceed; errors inline</v>
+      </c>
+    </row>
+    <row r="135" xml:space="preserve">
+      <c r="A135" t="str">
+        <v>S6M-40</v>
+      </c>
+      <c r="B135" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C135" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E135" t="str">
+        <v>UX consistency</v>
+      </c>
+      <c r="F135" t="str">
+        <v>As a Sales agent, I want consistent Marketing UI connected to CRM, so that the module feels enterprise-grade.</v>
+      </c>
+      <c r="G135" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H135">
+        <v>3</v>
+      </c>
+      <c r="I135" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J135" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K135" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Shared dashboard shell, typography, settings cards pattern
+• Breadcrumbs: Marketing → Campaigns → [name]
+• Contact links open CRM profile in same tab
+• QA pass on responsive breakpoints</v>
+      </c>
+    </row>
+    <row r="136" xml:space="preserve">
+      <c r="A136" t="str">
+        <v>S6M-41</v>
+      </c>
+      <c r="B136" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C136" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E136" t="str">
+        <v>Email sequence</v>
+      </c>
+      <c r="F136" t="str">
+        <v>As a Sales agent, I want mandatory merge-field validation before launch, so that every email includes required personalization.</v>
+      </c>
+      <c r="G136" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H136">
+        <v>3</v>
+      </c>
+      <c r="I136" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J136" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K136" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Each step body must include {{first_name}}
+• If {{contact_message}} appears in subject/body, source mode must be configured for that step (S6M-19)
+• {{phone}} and empty {{contact_message}} omitted in output when absent (no literal empty token)
+• Validation errors list all steps before launch</v>
+      </c>
+    </row>
+    <row r="137" xml:space="preserve">
+      <c r="A137" t="str">
+        <v>S6M-42</v>
+      </c>
+      <c r="B137" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C137" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E137" t="str">
+        <v>Stop rules</v>
+      </c>
+      <c r="F137" t="str">
+        <v>As a Platform, I want the send engine to skip stopped recipients before each step, so that cancelled follow-ups never dispatch.</v>
+      </c>
+      <c r="G137" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H137">
+        <v>3</v>
+      </c>
+      <c r="I137" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J137" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K137" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Before send: if campaign_recipient.stopped_reason is set, skip all pending steps (mark status=skipped, reason copied to activity log)
+• Cron idempotent check respects stopped state
+• Stats and activity log record skip reason</v>
+      </c>
+    </row>
+    <row r="138" xml:space="preserve">
+      <c r="A138" t="str">
+        <v>S6M-43</v>
+      </c>
+      <c r="B138" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C138" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D138" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Analytics</v>
+      </c>
+      <c r="F138" t="str">
+        <v>As a Sales agent, I want a per-recipient per-email-step detail view, so that I can see exactly what happened for each follow-up.</v>
+      </c>
+      <c r="G138" t="str">
+        <v>Agent</v>
+      </c>
+      <c r="H138">
+        <v>5</v>
+      </c>
+      <c r="I138" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J138" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K138" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Recipient row expands or drill-down shows each step: scheduled time, sent time, delivered, opened, clicked, step status, stopped_reason (recipient-level if stopped)
+• Links to provider message id (admin)
+• Matches contact profile timeline events</v>
+      </c>
+    </row>
+    <row r="139" xml:space="preserve">
+      <c r="A139" t="str">
+        <v>S6M-44</v>
+      </c>
+      <c r="B139" t="str">
+        <v>S6M</v>
+      </c>
+      <c r="C139" t="str">
+        <v>Marketing Campaign Redesign</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Planned 2026-Q3</v>
+      </c>
+      <c r="E139" t="str">
+        <v>Stop rules</v>
+      </c>
+      <c r="F139" t="str">
+        <v>As a Platform, I want spam complaints to stop remaining follow-ups and suppress the address globally, so that deliverability matches ESP industry practice.</v>
+      </c>
+      <c r="G139" t="str">
+        <v>Platform</v>
+      </c>
+      <c r="H139">
+        <v>3</v>
+      </c>
+      <c r="I139" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J139" t="str">
+        <v>Planned</v>
+      </c>
+      <c r="K139" t="str" xml:space="preserve">
+        <v xml:space="preserve">• On complained webhook: global suppress + campaign_recipient.stopped_reason=complaint
+• Pending steps status=stopped_complaint for that campaign only (same as hard bounce)
+• Admin alert or activity log entry for complaint events
+• Stats aggregate stopped_complaint count</v>
+      </c>
+    </row>
+    <row r="140" xml:space="preserve">
+      <c r="A140" t="str">
         <v>S7B-1</v>
       </c>
-      <c r="B96" t="str">
+      <c r="B140" t="str">
         <v>S7B</v>
       </c>
-      <c r="C96" t="str">
+      <c r="C140" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D96" t="str">
+      <c r="D140" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E96" t="str">
+      <c r="E140" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F96" t="str">
+      <c r="F140" t="str">
         <v>As a Admin, I want tenant-owned API credentials stored encrypted, so that email and AI providers use our keys securely.</v>
       </c>
-      <c r="G96" t="str">
+      <c r="G140" t="str">
         <v>Admin</v>
       </c>
-      <c r="H96">
-        <v>5</v>
-      </c>
-      <c r="I96" t="str">
-        <v>Must</v>
-      </c>
-      <c r="J96" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K96" t="str" xml:space="preserve">
+      <c r="H140">
+        <v>5</v>
+      </c>
+      <c r="I140" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J140" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K140" t="str" xml:space="preserve">
         <v xml:space="preserve">• account_service_credentials with AES-256-GCM encryption
 • secret_prefix masking in UI; plaintext never returned from API</v>
       </c>
     </row>
-    <row r="97" xml:space="preserve">
-      <c r="A97" t="str">
+    <row r="141" xml:space="preserve">
+      <c r="A141" t="str">
         <v>S7B-2</v>
       </c>
-      <c r="B97" t="str">
+      <c r="B141" t="str">
         <v>S7B</v>
       </c>
-      <c r="C97" t="str">
+      <c r="C141" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D97" t="str">
+      <c r="D141" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E97" t="str">
+      <c r="E141" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F97" t="str">
+      <c r="F141" t="str">
         <v>As a Admin, I want a Connected services settings page to manage email, AI, and enrichment providers.</v>
       </c>
-      <c r="G97" t="str">
+      <c r="G141" t="str">
         <v>Admin</v>
       </c>
-      <c r="H97">
+      <c r="H141">
         <v>3</v>
       </c>
-      <c r="I97" t="str">
-        <v>Must</v>
-      </c>
-      <c r="J97" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K97" t="str" xml:space="preserve">
+      <c r="I141" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J141" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K141" t="str" xml:space="preserve">
         <v xml:space="preserve">• Settings → Connected services lists connections by category
 • Add, edit, test, remove, set default per category</v>
       </c>
     </row>
-    <row r="98" xml:space="preserve">
-      <c r="A98" t="str">
+    <row r="142" xml:space="preserve">
+      <c r="A142" t="str">
         <v>S7B-3</v>
       </c>
-      <c r="B98" t="str">
+      <c r="B142" t="str">
         <v>S7B</v>
       </c>
-      <c r="C98" t="str">
+      <c r="C142" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D98" t="str">
+      <c r="D142" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E98" t="str">
+      <c r="E142" t="str">
         <v/>
       </c>
-      <c r="F98" t="str">
+      <c r="F142" t="str">
         <v>As a Marketer, I want marketing emails sent via my connected Resend (or other ESP) key.</v>
       </c>
-      <c r="G98" t="str">
+      <c r="G142" t="str">
         <v>Marketer</v>
       </c>
-      <c r="H98">
-        <v>5</v>
-      </c>
-      <c r="I98" t="str">
-        <v>Must</v>
-      </c>
-      <c r="J98" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K98" t="str" xml:space="preserve">
+      <c r="H142">
+        <v>5</v>
+      </c>
+      <c r="I142" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J142" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K142" t="str" xml:space="preserve">
         <v xml:space="preserve">• Resend verify + send adapter
 • Optional domain check for from-address</v>
       </c>
     </row>
-    <row r="99" xml:space="preserve">
-      <c r="A99" t="str">
+    <row r="143" xml:space="preserve">
+      <c r="A143" t="str">
         <v>S7B-4</v>
       </c>
-      <c r="B99" t="str">
+      <c r="B143" t="str">
         <v>S7B</v>
       </c>
-      <c r="C99" t="str">
+      <c r="C143" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D99" t="str">
+      <c r="D143" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E99" t="str">
+      <c r="E143" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F99" t="str">
+      <c r="F143" t="str">
         <v>As a Admin, I want SendGrid and Mailgun as alternate email providers.</v>
       </c>
-      <c r="G99" t="str">
+      <c r="G143" t="str">
         <v>Admin</v>
       </c>
-      <c r="H99">
-        <v>5</v>
-      </c>
-      <c r="I99" t="str">
+      <c r="H143">
+        <v>5</v>
+      </c>
+      <c r="I143" t="str">
         <v>Should</v>
       </c>
-      <c r="J99" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K99" t="str" xml:space="preserve">
+      <c r="J143" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K143" t="str" xml:space="preserve">
         <v xml:space="preserve">• Provider adapters with verify + send
 • Mailgun requires sending domain in config</v>
       </c>
     </row>
-    <row r="100" xml:space="preserve">
-      <c r="A100" t="str">
+    <row r="144" xml:space="preserve">
+      <c r="A144" t="str">
         <v>S7B-5</v>
       </c>
-      <c r="B100" t="str">
+      <c r="B144" t="str">
         <v>S7B</v>
       </c>
-      <c r="C100" t="str">
+      <c r="C144" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D100" t="str">
+      <c r="D144" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E100" t="str">
+      <c r="E144" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F100" t="str">
+      <c r="F144" t="str">
         <v>As a Marketer, I want each sender to use a specific connected credential.</v>
       </c>
-      <c r="G100" t="str">
+      <c r="G144" t="str">
         <v>Marketer</v>
       </c>
-      <c r="H100">
+      <c r="H144">
         <v>3</v>
       </c>
-      <c r="I100" t="str">
-        <v>Must</v>
-      </c>
-      <c r="J100" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K100" t="str" xml:space="preserve">
+      <c r="I144" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J144" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K144" t="str" xml:space="preserve">
         <v xml:space="preserve">• marketing_senders.credential_id FK
 • Send path resolves sender credential or account default</v>
       </c>
     </row>
-    <row r="101" xml:space="preserve">
-      <c r="A101" t="str">
+    <row r="145" xml:space="preserve">
+      <c r="A145" t="str">
         <v>S7B-6</v>
       </c>
-      <c r="B101" t="str">
+      <c r="B145" t="str">
         <v>S7B</v>
       </c>
-      <c r="C101" t="str">
+      <c r="C145" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D101" t="str">
+      <c r="D145" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E101" t="str">
+      <c r="E145" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F101" t="str">
+      <c r="F145" t="str">
         <v>As a Admin, I want per-credential webhook URLs for email delivery events.</v>
       </c>
-      <c r="G101" t="str">
+      <c r="G145" t="str">
         <v>Admin</v>
       </c>
-      <c r="H101">
+      <c r="H145">
         <v>3</v>
       </c>
-      <c r="I101" t="str">
-        <v>Must</v>
-      </c>
-      <c r="J101" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K101" t="str" xml:space="preserve">
+      <c r="I145" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J145" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K145" t="str" xml:space="preserve">
         <v xml:space="preserve">• POST /api/webhooks/email/[credentialId] with signature verification
 • Events update campaign recipient status</v>
       </c>
     </row>
-    <row r="102" xml:space="preserve">
-      <c r="A102" t="str">
+    <row r="146" xml:space="preserve">
+      <c r="A146" t="str">
         <v>S7B-7</v>
       </c>
-      <c r="B102" t="str">
+      <c r="B146" t="str">
         <v>S7B</v>
       </c>
-      <c r="C102" t="str">
+      <c r="C146" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D102" t="str">
+      <c r="D146" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E102" t="str">
+      <c r="E146" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F102" t="str">
+      <c r="F146" t="str">
         <v>As a Admin, I want Anthropic BYOK for widget AI replies.</v>
       </c>
-      <c r="G102" t="str">
+      <c r="G146" t="str">
         <v>Admin</v>
       </c>
-      <c r="H102">
-        <v>5</v>
-      </c>
-      <c r="I102" t="str">
+      <c r="H146">
+        <v>5</v>
+      </c>
+      <c r="I146" t="str">
         <v>Should</v>
       </c>
-      <c r="J102" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K102" t="str" xml:space="preserve">
+      <c r="J146" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K146" t="str" xml:space="preserve">
         <v xml:space="preserve">• AI chat proxy route uses tenant credential
 • Widget AI toggle in Connected services</v>
       </c>
     </row>
-    <row r="103" xml:space="preserve">
-      <c r="A103" t="str">
+    <row r="147" xml:space="preserve">
+      <c r="A147" t="str">
         <v>S7B-8</v>
       </c>
-      <c r="B103" t="str">
+      <c r="B147" t="str">
         <v>S7B</v>
       </c>
-      <c r="C103" t="str">
+      <c r="C147" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D103" t="str">
+      <c r="D147" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E103" t="str">
+      <c r="E147" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F103" t="str">
+      <c r="F147" t="str">
         <v>As a Admin, I want audit logs when service credentials are created, updated, or deleted.</v>
       </c>
-      <c r="G103" t="str">
+      <c r="G147" t="str">
         <v>Admin</v>
       </c>
-      <c r="H103">
+      <c r="H147">
         <v>3</v>
       </c>
-      <c r="I103" t="str">
-        <v>Must</v>
-      </c>
-      <c r="J103" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K103" t="str" xml:space="preserve">
+      <c r="I147" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J147" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K147" t="str" xml:space="preserve">
         <v xml:space="preserve">• Administrator-only credential CRUD
 • Test connection updates status and last_verified_at</v>
       </c>
     </row>
-    <row r="104" xml:space="preserve">
-      <c r="A104" t="str">
+    <row r="148" xml:space="preserve">
+      <c r="A148" t="str">
         <v>S7B-9</v>
       </c>
-      <c r="B104" t="str">
+      <c r="B148" t="str">
         <v>S7B</v>
       </c>
-      <c r="C104" t="str">
+      <c r="C148" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D104" t="str">
+      <c r="D148" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E104" t="str">
+      <c r="E148" t="str">
         <v>Connected Services</v>
       </c>
-      <c r="F104" t="str">
+      <c r="F148" t="str">
         <v>As a Admin, I want a workspace policy to require tenant email credentials (disable platform Resend fallback).</v>
       </c>
-      <c r="G104" t="str">
+      <c r="G148" t="str">
         <v>Admin</v>
       </c>
-      <c r="H104">
+      <c r="H148">
         <v>3</v>
       </c>
-      <c r="I104" t="str">
+      <c r="I148" t="str">
         <v>Should</v>
       </c>
-      <c r="J104" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K104" t="str" xml:space="preserve">
+      <c r="J148" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K148" t="str" xml:space="preserve">
         <v xml:space="preserve">• marketingByokOnly account setting
 • Sends blocked with clear message when no tenant ESP configured</v>
       </c>
     </row>
-    <row r="105" xml:space="preserve">
-      <c r="A105" t="str">
+    <row r="149" xml:space="preserve">
+      <c r="A149" t="str">
         <v>S7B-10</v>
       </c>
-      <c r="B105" t="str">
+      <c r="B149" t="str">
         <v>S7B</v>
       </c>
-      <c r="C105" t="str">
+      <c r="C149" t="str">
         <v>Connected Services (BYOK)</v>
       </c>
-      <c r="D105" t="str">
+      <c r="D149" t="str">
         <v>Implemented 2026-06</v>
       </c>
-      <c r="E105" t="str">
+      <c r="E149" t="str">
         <v>Connected Services — Enrichment</v>
       </c>
-      <c r="F105" t="str">
+      <c r="F149" t="str">
         <v>As a Admin, I want data enrichment providers in Connected services alongside email and AI, so that enrichment BYOK is discoverable in one place.</v>
       </c>
-      <c r="G105" t="str">
+      <c r="G149" t="str">
         <v>Admin</v>
       </c>
-      <c r="H105">
+      <c r="H149">
         <v>3</v>
       </c>
-      <c r="I105" t="str">
-        <v>Must</v>
-      </c>
-      <c r="J105" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="K105" t="str" xml:space="preserve">
+      <c r="I149" t="str">
+        <v>Must</v>
+      </c>
+      <c r="J149" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="K149" t="str" xml:space="preserve">
         <v xml:space="preserve">• Data enrichment section in Settings → Connected services
 • Provider list matches S6-26 adapters; test connection and usage counters
 • Extends encrypted credential store from S7B-1</v>
@@ -4437,14 +6080,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K149"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4630,59 +6273,85 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>S7B</v>
+        <v>S6M</v>
       </c>
       <c r="B8" t="str">
-        <v>Connected Services (BYOK)</v>
+        <v>Marketing Campaign Redesign</v>
       </c>
       <c r="C8" t="str">
-        <v>Implemented 2026-06</v>
+        <v>Planned 2026-Q3</v>
       </c>
       <c r="D8">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="E8">
-        <v>38</v>
+        <v>185</v>
       </c>
       <c r="F8">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="G8">
         <v>3</v>
       </c>
       <c r="H8" t="str">
-        <v>✅ Completed</v>
+        <v>📋 Planned</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>S7B</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Connected Services (BYOK)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Implemented 2026-06</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>38</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
+      </c>
+      <c r="H9" t="str">
+        <v>✅ Completed</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B10" t="str">
         <v/>
       </c>
-      <c r="C9" t="str">
+      <c r="C10" t="str">
         <v/>
       </c>
-      <c r="D9">
-        <v>104</v>
-      </c>
-      <c r="E9">
-        <v>491</v>
-      </c>
-      <c r="F9" t="str">
+      <c r="D10">
+        <v>148</v>
+      </c>
+      <c r="E10">
+        <v>676</v>
+      </c>
+      <c r="F10" t="str">
         <v/>
       </c>
-      <c r="G9" t="str">
+      <c r="G10" t="str">
         <v/>
       </c>
-      <c r="H9" t="str">
+      <c r="H10" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ship S7–S20 platform scaffolding, security hardening, and headless chat mode.
Add hosted/headless widget mode (default hosted for existing tenants), channel/automation/AI/help-center APIs and settings UI, webhook and cron fail-closed auth, and related product docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/FlowChat_User_Stories_S1_S6.xlsx
+++ b/FlowChat_User_Stories_S1_S6.xlsx
@@ -3571,7 +3571,7 @@
       <c r="K82" t="str" xml:space="preserve">
         <v xml:space="preserve">• [Superseded by S6M — see marketing-module-screens.md] Was: visual workflow builder with CRM triggers (contact created, label added, conversation resolved)
 • Replacement: campaign-only wizard with explicit recipients (S6M-6, S6M-9)
-• Remove triggerMarketingWorkflows at S6M-9 implementation</v>
+• Remove triggerMarketingWorkflows at S6M-9 closeout (still Partial in codebase as of 2026-07-25)</v>
       </c>
     </row>
     <row r="83" xml:space="preserve">
@@ -4079,7 +4079,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D96" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E96" t="str">
         <v>Campaign lifecycle</v>
@@ -4097,7 +4097,7 @@
         <v>Must</v>
       </c>
       <c r="J96" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K96" t="str" xml:space="preserve">
         <v xml:space="preserve">• Wizard step 0 saves draft via POST /marketing/campaigns
@@ -4117,7 +4117,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D97" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E97" t="str">
         <v>Campaign lifecycle</v>
@@ -4135,7 +4135,7 @@
         <v>Must</v>
       </c>
       <c r="J97" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K97" t="str" xml:space="preserve">
         <v xml:space="preserve">• Marketing home lists campaigns with status badges: draft, scheduled, running, paused, completed, cancelled
@@ -4154,7 +4154,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D98" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E98" t="str">
         <v>Campaign lifecycle</v>
@@ -4172,7 +4172,7 @@
         <v>Must</v>
       </c>
       <c r="J98" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K98" t="str" xml:space="preserve">
         <v xml:space="preserve">• Only administrator role can launch
@@ -4193,7 +4193,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D99" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E99" t="str">
         <v>Campaign lifecycle</v>
@@ -4211,7 +4211,7 @@
         <v>Must</v>
       </c>
       <c r="J99" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K99" t="str" xml:space="preserve">
         <v xml:space="preserve">• Pause stops new sends; in-flight batch completes
@@ -4231,7 +4231,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D100" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E100" t="str">
         <v>Campaign lifecycle</v>
@@ -4249,7 +4249,7 @@
         <v>Should</v>
       </c>
       <c r="J100" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K100" t="str" xml:space="preserve">
         <v xml:space="preserve">• Duplicate copies steps and templates (snapshot) not live template links
@@ -4268,7 +4268,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D101" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E101" t="str">
         <v>Recipients</v>
@@ -4286,7 +4286,7 @@
         <v>Must</v>
       </c>
       <c r="J101" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K101" t="str" xml:space="preserve">
         <v xml:space="preserve">• Step 1: search CRM contacts with email
@@ -4306,7 +4306,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D102" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E102" t="str">
         <v>Recipients</v>
@@ -4324,7 +4324,7 @@
         <v>Should</v>
       </c>
       <c r="J102" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K102" t="str" xml:space="preserve">
         <v xml:space="preserve">• Optional “Import from segment” on step 1
@@ -4343,7 +4343,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D103" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E103" t="str">
         <v>Recipients</v>
@@ -4361,7 +4361,7 @@
         <v>Must</v>
       </c>
       <c r="J103" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K103" t="str" xml:space="preserve">
         <v xml:space="preserve">• Suppressed/unsubscribed/bounced contacts flagged in picker
@@ -4380,7 +4380,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D104" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E104" t="str">
         <v>CRM isolation</v>
@@ -4398,13 +4398,14 @@
         <v>Must</v>
       </c>
       <c r="J104" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K104" t="str" xml:space="preserve">
         <v xml:space="preserve">• Remove triggerMarketingWorkflows on contact_created from: manual CRUD, CSV import, LeadSnapper/integration upsert, widget session create
 • Remove conversation_resolved and label_added auto-enroll from marketing
 • Legacy workflow UI hidden or admin-only deprecated
-• CRM contacts unaffected when added via any medium; double opt-in transactional mail is not a marketing campaign</v>
+• CRM contacts unaffected when added via any medium; double opt-in transactional mail is not a marketing campaign
+• [Codebase 2026-07-25] COMPLETED — call sites removed; function is no-op; Lead Monitor/LeadSnapper sync does not enroll marketing</v>
       </c>
     </row>
     <row r="105" xml:space="preserve">
@@ -4418,7 +4419,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D105" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E105" t="str">
         <v>Recipients</v>
@@ -4436,7 +4437,7 @@
         <v>Must</v>
       </c>
       <c r="J105" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K105" t="str" xml:space="preserve">
         <v xml:space="preserve">• Step 4 lists recipient names and emails (paginated)
@@ -4455,7 +4456,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D106" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E106" t="str">
         <v>Templates</v>
@@ -4473,7 +4474,7 @@
         <v>Must</v>
       </c>
       <c r="J106" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K106" t="str" xml:space="preserve">
         <v xml:space="preserve">• Marketing → Templates: list, create, edit, archive, duplicate
@@ -4492,7 +4493,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D107" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E107" t="str">
         <v>Templates</v>
@@ -4510,7 +4511,7 @@
         <v>Must</v>
       </c>
       <c r="J107" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K107" t="str" xml:space="preserve">
         <v xml:space="preserve">• Composer opens full viewport overlay from wizard or template library
@@ -4531,7 +4532,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D108" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E108" t="str">
         <v>Templates</v>
@@ -4549,7 +4550,7 @@
         <v>Must</v>
       </c>
       <c r="J108" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K108" t="str" xml:space="preserve">
         <v xml:space="preserve">• Per sequence step: “Save as template” with name field
@@ -4568,7 +4569,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D109" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E109" t="str">
         <v>Templates</v>
@@ -4586,7 +4587,7 @@
         <v>Must</v>
       </c>
       <c r="J109" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K109" t="str" xml:space="preserve">
         <v xml:space="preserve">• campaign_steps store subject/html snapshot per step
@@ -4605,7 +4606,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D110" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E110" t="str">
         <v>Templates</v>
@@ -4623,7 +4624,7 @@
         <v>Must</v>
       </c>
       <c r="J110" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K110" t="str" xml:space="preserve">
         <v xml:space="preserve">• Chips: first_name, last_name, email, phone, contact_message, meeting_link, portfolio_link, agent_name, agent_email
@@ -4642,7 +4643,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D111" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E111" t="str">
         <v>Email sequence</v>
@@ -4660,7 +4661,7 @@
         <v>Must</v>
       </c>
       <c r="J111" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K111" t="str" xml:space="preserve">
         <v xml:space="preserve">• Step 2: add/remove email rows (min 1)
@@ -4680,7 +4681,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D112" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E112" t="str">
         <v>Email sequence</v>
@@ -4698,7 +4699,7 @@
         <v>Must</v>
       </c>
       <c r="J112" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K112" t="str" xml:space="preserve">
         <v xml:space="preserve">• Date+time picker per step; no system timezone preference for scheduling UI
@@ -4717,7 +4718,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D113" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E113" t="str">
         <v>Email sequence</v>
@@ -4735,7 +4736,7 @@
         <v>Must</v>
       </c>
       <c r="J113" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K113" t="str" xml:space="preserve">
         <v xml:space="preserve">• Step N send_at &gt; step N-1 send_at
@@ -4754,7 +4755,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D114" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E114" t="str">
         <v>Email sequence</v>
@@ -4772,7 +4773,7 @@
         <v>Must</v>
       </c>
       <c r="J114" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K114" t="str" xml:space="preserve">
         <v xml:space="preserve">• Per step with {{contact_message}}: agent selects source mode (industry-standard per-recipient resolution):
@@ -4795,7 +4796,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D115" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E115" t="str">
         <v>Email sequence</v>
@@ -4813,7 +4814,7 @@
         <v>Must</v>
       </c>
       <c r="J115" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K115" t="str" xml:space="preserve">
         <v xml:space="preserve">• No attachment UI in composer
@@ -4832,7 +4833,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D116" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E116" t="str">
         <v>Signature &amp; compliance</v>
@@ -4850,7 +4851,7 @@
         <v>Must</v>
       </c>
       <c r="J116" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K116" t="str" xml:space="preserve">
         <v xml:space="preserve">• Step 3: signature rich editor or workspace default
@@ -4869,7 +4870,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D117" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E117" t="str">
         <v>Signature &amp; compliance</v>
@@ -4887,7 +4888,7 @@
         <v>Must</v>
       </c>
       <c r="J117" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K117" t="str" xml:space="preserve">
         <v xml:space="preserve">• meeting_link and portfolio_link merge tags from workspace settings; overridable per campaign
@@ -4906,7 +4907,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D118" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E118" t="str">
         <v>Signature &amp; compliance</v>
@@ -4924,7 +4925,7 @@
         <v>Must</v>
       </c>
       <c r="J118" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K118" t="str" xml:space="preserve">
         <v xml:space="preserve">• Launch button disabled until a test send succeeded for this campaign draft (persists across sessions until content/sender changes invalidate)
@@ -4943,7 +4944,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D119" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E119" t="str">
         <v>Infrastructure</v>
@@ -4961,7 +4962,7 @@
         <v>Must</v>
       </c>
       <c r="J119" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K119" t="str" xml:space="preserve">
         <v xml:space="preserve">• Checks: connected Resend/SendGrid/Mailgun or platform key; domain verified; last cron success &lt; 2 min
@@ -4980,7 +4981,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D120" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E120" t="str">
         <v>Signature &amp; compliance</v>
@@ -4998,7 +4999,7 @@
         <v>Must</v>
       </c>
       <c r="J120" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K120" t="str" xml:space="preserve">
         <v xml:space="preserve">• System appends List-Unsubscribe header and footer link
@@ -5017,7 +5018,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D121" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E121" t="str">
         <v>Analytics</v>
@@ -5035,7 +5036,7 @@
         <v>Must</v>
       </c>
       <c r="J121" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K121" t="str" xml:space="preserve">
         <v xml:space="preserve">• Detail page: sent, delivered, opened, clicked, bounced, unsubscribed, complained, stopped counts
@@ -5055,7 +5056,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D122" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E122" t="str">
         <v>Analytics</v>
@@ -5073,7 +5074,7 @@
         <v>Must</v>
       </c>
       <c r="J122" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K122" t="str" xml:space="preserve">
         <v xml:space="preserve">• Tab or section per step: subject, scheduled time, sent count, open %, click %
@@ -5091,7 +5092,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D123" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E123" t="str">
         <v>Analytics</v>
@@ -5109,7 +5110,7 @@
         <v>Must</v>
       </c>
       <c r="J123" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K123" t="str" xml:space="preserve">
         <v xml:space="preserve">• Columns: contact, email, per-step status, stopped_reason, last event time
@@ -5128,7 +5129,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D124" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E124" t="str">
         <v>Analytics</v>
@@ -5146,7 +5147,7 @@
         <v>Should</v>
       </c>
       <c r="J124" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K124" t="str" xml:space="preserve">
         <v xml:space="preserve">• Export recipient × step × status × timestamps
@@ -5165,7 +5166,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D125" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E125" t="str">
         <v>Analytics</v>
@@ -5183,7 +5184,7 @@
         <v>Must</v>
       </c>
       <c r="J125" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K125" t="str" xml:space="preserve">
         <v xml:space="preserve">• Contact profile shows campaign name, step, sent/opened/clicked/stopped events
@@ -5201,7 +5202,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D126" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E126" t="str">
         <v>Infrastructure</v>
@@ -5219,7 +5220,7 @@
         <v>Must</v>
       </c>
       <c r="J126" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K126" t="str" xml:space="preserve">
         <v xml:space="preserve">• MarketingError codes mapped to UI strings per §3.1 marketing-module-screens.md
@@ -5238,7 +5239,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D127" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E127" t="str">
         <v>Infrastructure</v>
@@ -5256,7 +5257,7 @@
         <v>Must</v>
       </c>
       <c r="J127" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K127" t="str" xml:space="preserve">
         <v xml:space="preserve">• Agents can build drafts; launch requires administrator role
@@ -5275,7 +5276,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D128" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E128" t="str">
         <v>Infrastructure</v>
@@ -5293,7 +5294,7 @@
         <v>Must</v>
       </c>
       <c r="J128" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K128" t="str" xml:space="preserve">
         <v xml:space="preserve">• job-runner processes campaign_recipient_steps where send_at &lt;= now
@@ -5314,7 +5315,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D129" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E129" t="str">
         <v>Infrastructure</v>
@@ -5332,7 +5333,7 @@
         <v>Must</v>
       </c>
       <c r="J129" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K129" t="str" xml:space="preserve">
         <v xml:space="preserve">• Per-credential webhook URLs ingest delivered, opened, clicked, bounced, complained
@@ -5351,7 +5352,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D130" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E130" t="str">
         <v>CRM isolation</v>
@@ -5369,7 +5370,7 @@
         <v>Must</v>
       </c>
       <c r="J130" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K130" t="str" xml:space="preserve">
         <v xml:space="preserve">• Nav: Campaigns, Templates only (segments optional sub-link)
@@ -5388,7 +5389,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D131" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E131" t="str">
         <v>Stop rules</v>
@@ -5406,7 +5407,7 @@
         <v>Must</v>
       </c>
       <c r="J131" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K131" t="str" xml:space="preserve">
         <v xml:space="preserve">• Hard/permanent bounce (provider permanent flag or second soft within 72h): campaign_recipient.stopped_reason=bounce; pending steps set status=stopped_bounce
@@ -5427,7 +5428,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D132" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E132" t="str">
         <v>Stop rules</v>
@@ -5445,7 +5446,7 @@
         <v>Must</v>
       </c>
       <c r="J132" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K132" t="str" xml:space="preserve">
         <v xml:space="preserve">• Unsubscribe link suppresses globally and stops pending campaign steps for that address
@@ -5464,7 +5465,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D133" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E133" t="str">
         <v>Stop rules</v>
@@ -5482,14 +5483,15 @@
         <v>Must</v>
       </c>
       <c r="J133" t="str">
-        <v>Planned</v>
+        <v>Partial</v>
       </c>
       <c r="K133" t="str" xml:space="preserve">
         <v xml:space="preserve">• Primary: inbound reply matched via In-Reply-To/References to outbound Message-ID (Sprint 7 email inbox)
 • Fallback until inbox live: provider reply/engagement webhook if supported by connected ESP
 • campaign_recipient.stopped_reason=reply; pending steps status=stopped_reply
 • Reply does not stop other campaigns or other recipients
-• Documented dependency: full reply-stop requires Sprint 7 inbound routing</v>
+• Documented dependency: full reply-stop requires Sprint 7 inbound routing
+• [Codebase 2026-07-25] PARTIAL — ESP reply webhook fallback only; blocked on Sprint 7 IMAP/thread continuity for full fidelity</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -5503,7 +5505,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D134" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E134" t="str">
         <v>Campaign lifecycle</v>
@@ -5521,7 +5523,7 @@
         <v>Must</v>
       </c>
       <c r="J134" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K134" t="str" xml:space="preserve">
         <v xml:space="preserve">• Steps: Recipients → Sequence → Sender → Review
@@ -5540,7 +5542,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D135" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E135" t="str">
         <v>UX consistency</v>
@@ -5558,7 +5560,7 @@
         <v>Must</v>
       </c>
       <c r="J135" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K135" t="str" xml:space="preserve">
         <v xml:space="preserve">• Shared dashboard shell, typography, settings cards pattern
@@ -5578,7 +5580,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D136" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E136" t="str">
         <v>Email sequence</v>
@@ -5596,7 +5598,7 @@
         <v>Must</v>
       </c>
       <c r="J136" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K136" t="str" xml:space="preserve">
         <v xml:space="preserve">• Each step body must include {{first_name}}
@@ -5616,7 +5618,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D137" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E137" t="str">
         <v>Stop rules</v>
@@ -5634,7 +5636,7 @@
         <v>Must</v>
       </c>
       <c r="J137" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K137" t="str" xml:space="preserve">
         <v xml:space="preserve">• Before send: if campaign_recipient.stopped_reason is set, skip all pending steps (mark status=skipped, reason copied to activity log)
@@ -5653,7 +5655,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D138" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E138" t="str">
         <v>Analytics</v>
@@ -5671,7 +5673,7 @@
         <v>Must</v>
       </c>
       <c r="J138" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K138" t="str" xml:space="preserve">
         <v xml:space="preserve">• Recipient row expands or drill-down shows each step: scheduled time, sent time, delivered, opened, clicked, step status, stopped_reason (recipient-level if stopped)
@@ -5690,7 +5692,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D139" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E139" t="str">
         <v>Stop rules</v>
@@ -5708,7 +5710,7 @@
         <v>Must</v>
       </c>
       <c r="J139" t="str">
-        <v>Planned</v>
+        <v>Completed</v>
       </c>
       <c r="K139" t="str" xml:space="preserve">
         <v xml:space="preserve">• On complained webhook: global suppress + campaign_recipient.stopped_reason=complaint
@@ -5728,7 +5730,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="D140" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="E140" t="str">
         <v>Visual design</v>
@@ -6319,7 +6321,7 @@
         <v>Marketing Campaign Redesign</v>
       </c>
       <c r="C8" t="str">
-        <v>Planned 2026-Q3</v>
+        <v>Implemented 2026-Q2/Q3 — pending QA / closeout</v>
       </c>
       <c r="D8">
         <v>45</v>
@@ -6334,7 +6336,7 @@
         <v>4</v>
       </c>
       <c r="H8" t="str">
-        <v>📋 Planned</v>
+        <v>🟡 Implemented — pending QA / closeout</v>
       </c>
     </row>
     <row r="9">

</xml_diff>